<commit_message>
Use Fabric-compatible KYC branch scoping
</commit_message>
<xml_diff>
--- a/Ale-InspectionSuccursales.xlsx
+++ b/Ale-InspectionSuccursales.xlsx
@@ -8,15 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://peakgroup0-my.sharepoint.com/personal/aduplaga_peakgroup_com/Documents/source/repos/Compliance_BRN_Samples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="67" documentId="8_{C08D7061-467F-49D9-BA49-F53AFEEB14EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DD8A2B7-38B4-4EAD-82B6-0193990170E2}"/>
+  <xr:revisionPtr revIDLastSave="78" documentId="8_{C08D7061-467F-49D9-BA49-F53AFEEB14EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{33A23365-2774-412C-88FA-F3F914DC20E5}"/>
   <bookViews>
-    <workbookView xWindow="15195" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{CD0190AD-07ED-4561-9762-79CFF99B3F22}"/>
+    <workbookView xWindow="16800" yWindow="-15255" windowWidth="24195" windowHeight="13620" activeTab="1" xr2:uid="{CD0190AD-07ED-4561-9762-79CFF99B3F22}"/>
   </bookViews>
   <sheets>
     <sheet name="Logique" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="3" r:id="rId2"/>
     <sheet name="Scripts" sheetId="2" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Sheet1!$A$4:$I$10</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -41,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="59">
   <si>
     <t>Analyse d'affaire - échantillonnage pour inspection des succursales SPP</t>
   </si>
@@ -323,6 +326,9 @@
   </si>
   <si>
     <t>Done</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                 </t>
   </si>
 </sst>
 </file>
@@ -473,6 +479,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -835,6 +845,9 @@
       <c r="B9" s="3" t="s">
         <v>5</v>
       </c>
+      <c r="C9" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="11" spans="1:3" ht="108" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
@@ -844,7 +857,7 @@
         <v>7</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="108" x14ac:dyDescent="0.35">
@@ -937,47 +950,37 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="9">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="D5" s="9" t="s">
-        <v>56</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="C5" s="11"/>
+      <c r="D5" s="9"/>
       <c r="E5" s="9"/>
-      <c r="F5" s="9" t="s">
-        <v>55</v>
-      </c>
+      <c r="F5" s="9"/>
       <c r="G5" s="11"/>
-      <c r="H5" s="9"/>
+      <c r="H5" s="9">
+        <v>1</v>
+      </c>
       <c r="I5" s="9" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="D6" s="9">
-        <v>30</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="G6" s="11"/>
+        <v>41</v>
+      </c>
+      <c r="C6" s="11"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="11" t="s">
+        <v>40</v>
+      </c>
       <c r="H6" s="9"/>
       <c r="I6" s="9" t="s">
         <v>49</v>
@@ -985,13 +988,13 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="D7" s="9"/>
       <c r="E7" s="9"/>
@@ -1006,13 +1009,13 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D8" s="9"/>
       <c r="E8" s="9"/>
@@ -1027,18 +1030,24 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="9">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="11" t="s">
-        <v>40</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="9">
+        <v>30</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="G9" s="11"/>
       <c r="H9" s="9"/>
       <c r="I9" s="9" t="s">
         <v>49</v>
@@ -1046,19 +1055,23 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="9">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" s="11"/>
-      <c r="D10" s="9"/>
+        <v>30</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>56</v>
+      </c>
       <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
+      <c r="F10" s="9" t="s">
+        <v>55</v>
+      </c>
       <c r="G10" s="11"/>
-      <c r="H10" s="9">
-        <v>1</v>
-      </c>
+      <c r="H10" s="9"/>
       <c r="I10" s="9" t="s">
         <v>49</v>
       </c>
@@ -1201,6 +1214,11 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A4:I10" xr:uid="{C9921D99-4432-40A9-A519-DF5B39DD0ABF}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A5:I10">
+      <sortCondition ref="A4:A10"/>
+    </sortState>
+  </autoFilter>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1277,12 +1295,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0ef1a97a-1525-4ed2-8a8e-361511404792">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="c0fd1c75-a352-4d68-8516-d309e31bea90" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1515,20 +1535,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0ef1a97a-1525-4ed2-8a8e-361511404792">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="c0fd1c75-a352-4d68-8516-d309e31bea90" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1A1D9A5-C798-4B8F-8C4B-30C2548BF16C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62DBD3C3-9991-4938-9B89-33B1DA4B502F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="0ef1a97a-1525-4ed2-8a8e-361511404792"/>
+    <ds:schemaRef ds:uri="c0fd1c75-a352-4d68-8516-d309e31bea90"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1553,12 +1574,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62DBD3C3-9991-4938-9B89-33B1DA4B502F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1A1D9A5-C798-4B8F-8C4B-30C2548BF16C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="0ef1a97a-1525-4ed2-8a8e-361511404792"/>
-    <ds:schemaRef ds:uri="c0fd1c75-a352-4d68-8516-d309e31bea90"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>